<commit_message>
feat: add pre-API validation for clan operations
- Add pre-API validation to create_clan, destroy_clan, join_clan_member, leave_clan_member, kick_clan_member, change_clan_role, set_clan_title
- Validate master cannot leave clan (must use destroy_clan)
- Validate destroy_clan requires master role and only one member
- Validate set_clan_title requires master role and title constraints
- Add exception handling with user-friendly error messages
- Split MESSAGE_CLAN_MEMBER_ACTION into MESSAGE_CLAN_MEMBER_KICKED and MESSAGE_CLAN_MEMBER_LEFT
- Add new message constants: MESSAGE_CLAN_NO_PRIVILEGE, MESSAGE_CLAN_CANNOT_LEAVE_MASTER, MESSAGE_CLAN_MEMBER_EXISTS, MESSAGE_CLAN_TITLE_NOT_CHANGED, MESSAGE_CLAN_TITLE_TOO_SHORT
- Update const.string.xlsx with new message constants
</commit_message>
<xml_diff>
--- a/resources/table/const.string.xlsx
+++ b/resources/table/const.string.xlsx
@@ -3883,7 +3883,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -3961,7 +3961,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_CLAN_MEMBER_ACTION</t>
+          <t>MESSAGE_CLAN_NO_PRIVILEGE</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -3976,14 +3976,14 @@
       </c>
       <c r="D4" s="1" t="inlineStr">
         <is>
-          <t>{}님이 문파에서 {}했습니다.</t>
+          <t>문파 권한이 부족합니다.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_CLAN_ROLE_CHANGED</t>
+          <t>MESSAGE_CLAN_CANNOT_LEAVE_MASTER</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -3998,14 +3998,14 @@
       </c>
       <c r="D5" s="1" t="inlineStr">
         <is>
-          <t>문파 직책이 변경되었습니다. ({} -&gt; {})</t>
+          <t>문파 마스터는 탈퇴할 수 없습니다.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_CLAN_DISBANDED</t>
+          <t>MESSAGE_CLAN_MEMBER_EXISTS</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -4020,14 +4020,14 @@
       </c>
       <c r="D6" s="1" t="inlineStr">
         <is>
-          <t>{} 문파가 해체되었습니다.</t>
+          <t>문파에 다른 멤버가 존재합니다.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_CLAN_MEMBER_JOINED</t>
+          <t>MESSAGE_CLAN_TITLE_NOT_CHANGED</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -4042,14 +4042,14 @@
       </c>
       <c r="D7" s="1" t="inlineStr">
         <is>
-          <t>{}님이 문파에 가입했습니다.</t>
+          <t>문파 칭호가 변경되지 않았습니다.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_CLAN_JOINED_SUCCESS</t>
+          <t>MESSAGE_CLAN_TITLE_TOO_SHORT</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -4064,27 +4064,159 @@
       </c>
       <c r="D8" s="1" t="inlineStr">
         <is>
-          <t>{} 문파에 가입되었습니다.</t>
+          <t>문파 칭호가 너무 짧습니다.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
+          <t>MESSAGE_CLAN_MEMBER_KICKED</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C9" s="1" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D9" s="1" t="inlineStr">
+        <is>
+          <t>{}님이 문파에서 추방당했습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>MESSAGE_CLAN_MEMBER_LEFT</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C10" s="1" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D10" s="1" t="inlineStr">
+        <is>
+          <t>{}님이 문파에서 탈퇴했습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>MESSAGE_CLAN_ROLE_CHANGED</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C11" s="1" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D11" s="1" t="inlineStr">
+        <is>
+          <t>문파 직책이 변경되었습니다. ({} -&gt; {})</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>MESSAGE_CLAN_DISBANDED</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C12" s="1" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D12" s="1" t="inlineStr">
+        <is>
+          <t>{} 문파가 해체되었습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>MESSAGE_CLAN_MEMBER_JOINED</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C13" s="1" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D13" s="1" t="inlineStr">
+        <is>
+          <t>{}님이 문파에 가입했습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>MESSAGE_CLAN_JOINED_SUCCESS</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C14" s="1" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D14" s="1" t="inlineStr">
+        <is>
+          <t>{} 문파에 가입되었습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
           <t>MESSAGE_CLAN_ROLE_CHANGED_DETAILED</t>
         </is>
       </c>
-      <c r="B9" s="1" t="inlineStr">
-        <is>
-          <t>server</t>
-        </is>
-      </c>
-      <c r="C9" s="1" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="D9" s="1" t="inlineStr">
+      <c r="B15" s="1" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C15" s="1" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D15" s="1" t="inlineStr">
         <is>
           <t>{}님의 문파 직책이 {}에서 {}로 변경되었습니다.</t>
         </is>

</xml_diff>

<commit_message>
feat: add marketplace message constants and improve dialog handling
- Add marketplace message constants to model.h string class
- Replace hardcoded English messages with localized constants in marketplace.cpp
- Replace hardcoded English messages with ConstValue.String constants in MarketplaceService.cs
- Add StringExtension.ToCSharpFormat() to convert C++ format strings to C# format
- Fix coroutine lifetime issues by copying id parameter in marketplace::cancel and purchase
- Update all me:dialog calls to enable PREV and NEXT buttons
- Implement return value propagation for QUIT/PREV/NEXT handling in handle_storage and handle_marketplace functions
- Fix SQL syntax error in UpdateListingStatusAsync
- Add JsonTypeHandler registrations for marketplace server Program.cs
</commit_message>
<xml_diff>
--- a/resources/table/const.string.xlsx
+++ b/resources/table/const.string.xlsx
@@ -4865,7 +4865,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D36"/>
+  <dimension ref="A1:D61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -5361,7 +5361,7 @@
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_NOT_ANY_REPAIRABLE</t>
+          <t>MESSAGE_MARKETPLACE_FAILED_ALLOCATE_LISTING_ID</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
@@ -5376,14 +5376,14 @@
       </c>
       <c r="D23" s="1" t="inlineStr">
         <is>
-          <t>고칠 물건이 없습니다.</t>
+          <t>거래소 등록 ID 할당에 실패했습니다. (에러코드: {})</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_CANNOT_DEPOSITE_MORE</t>
+          <t>MESSAGE_MARKETPLACE_CHARACTER_EXPIRED</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
@@ -5398,14 +5398,14 @@
       </c>
       <c r="D24" s="1" t="inlineStr">
         <is>
-          <t>더 이상 맡길 수 없습니다.</t>
+          <t>캐릭터가 만료되었습니다.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_NOT_DEPOSITED_MONEY</t>
+          <t>MESSAGE_MARKETPLACE_ITEM_NOT_FOUND_AT_INDEX</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
@@ -5420,14 +5420,14 @@
       </c>
       <c r="D25" s="1" t="inlineStr">
         <is>
-          <t>맡아둔 돈이 없습니다.</t>
+          <t>해당 인덱스에 아이템이 없습니다.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_NOT_DEPOSITED_ENOUGH</t>
+          <t>MESSAGE_MARKETPLACE_INSUFFICIENT_ITEM_COUNT</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
@@ -5442,14 +5442,14 @@
       </c>
       <c r="D26" s="1" t="inlineStr">
         <is>
-          <t>그만큼 맡기지 않았습니다.</t>
+          <t>아이템 수량이 부족합니다.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_HAVE_MUCH_MONEY</t>
+          <t>MESSAGE_MARKETPLACE_INSUFFICIENT_MONEY_FOR_LISTING_FEE</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
@@ -5464,14 +5464,14 @@
       </c>
       <c r="D27" s="1" t="inlineStr">
         <is>
-          <t>소지금이 너무 많습니다.</t>
+          <t>등록 수수료가 부족합니다.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_NOT_DEPOSITED_THIS_ITEM</t>
+          <t>MESSAGE_MARKETPLACE_FAILED_TO_LIST_ITEM</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
@@ -5486,14 +5486,14 @@
       </c>
       <c r="D28" s="1" t="inlineStr">
         <is>
-          <t>그런 물품은 맡아두고 있지 않습니다.</t>
+          <t>아이템 등록에 실패했습니다. (에러코드: {})</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_UNKNOWN_ERROR</t>
+          <t>MESSAGE_MARKETPLACE_FAILED_TO_LIST_ITEM_WITH_ERROR</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
@@ -5508,14 +5508,14 @@
       </c>
       <c r="D29" s="1" t="inlineStr">
         <is>
-          <t>알 수 없는 에러</t>
+          <t>아이템 등록에 실패했습니다. ({})</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_INVALID_ITEM_NAME</t>
+          <t>MESSAGE_MARKETPLACE_FAILED_TO_CANCEL_LISTING</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
@@ -5530,14 +5530,14 @@
       </c>
       <c r="D30" s="1" t="inlineStr">
         <is>
-          <t>그게 뭐야?</t>
+          <t>거래소 등록 취소에 실패했습니다. (에러코드: {})</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_WEAWPON_NAME_TOO_SHORT</t>
+          <t>MESSAGE_MARKETPLACE_LISTING_NOT_FOUND</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
@@ -5552,14 +5552,14 @@
       </c>
       <c r="D31" s="1" t="inlineStr">
         <is>
-          <t>이름이 너무 짧습니다.</t>
+          <t>등록된 물품을 찾을 수 없습니다.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_WEAPON_NAME_TOO_LONG</t>
+          <t>MESSAGE_MARKETPLACE_LISTING_NOT_AVAILABLE_FOR_PURCHASE</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -5574,14 +5574,14 @@
       </c>
       <c r="D32" s="1" t="inlineStr">
         <is>
-          <t>이름이 너무 깁니다.</t>
+          <t>구매할 수 없는 물품입니다.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_INVALID_WEAPON_NAME</t>
+          <t>MESSAGE_MARKETPLACE_INSUFFICIENT_MONEY</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
@@ -5596,14 +5596,14 @@
       </c>
       <c r="D33" s="1" t="inlineStr">
         <is>
-          <t>그렇게 바꿀 수 없습니다.</t>
+          <t>돈이 부족합니다.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_NO_ANY_DEPOSITED</t>
+          <t>MESSAGE_MARKETPLACE_FAILED_TO_PURCHASE_ITEM</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
@@ -5618,14 +5618,14 @@
       </c>
       <c r="D34" s="1" t="inlineStr">
         <is>
-          <t>맡긴 물건이 없습니다.</t>
+          <t>아이템 구매에 실패했습니다. (에러코드: {})</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_NO_ITEM_DEPOSITED</t>
+          <t>MESSAGE_MARKETPLACE_FAILED_TO_PURCHASE_ITEM_WITH_ERROR</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
@@ -5640,27 +5640,577 @@
       </c>
       <c r="D35" s="1" t="inlineStr">
         <is>
-          <t>그런 물건은 맡고 있지 않습니다.</t>
+          <t>아이템 구매에 실패했습니다. ({})</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
+          <t>MESSAGE_MARKETPLACE_FAILED_TO_SEARCH_ITEMS</t>
+        </is>
+      </c>
+      <c r="B36" s="1" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C36" s="1" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D36" s="1" t="inlineStr">
+        <is>
+          <t>아이템 검색에 실패했습니다. (에러코드: {})</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="inlineStr">
+        <is>
+          <t>MESSAGE_MARKETPLACE_FAILED_TO_GET_LISTINGS</t>
+        </is>
+      </c>
+      <c r="B37" s="1" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C37" s="1" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D37" s="1" t="inlineStr">
+        <is>
+          <t>등록 물품 조회에 실패했습니다. (에러코드: {})</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="inlineStr">
+        <is>
+          <t>MESSAGE_MARKETPLACE_LISTING_RECOVERY_TITLE</t>
+        </is>
+      </c>
+      <c r="B38" s="1" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C38" s="1" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D38" s="1" t="inlineStr">
+        <is>
+          <t>거래소 등록 복구</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="inlineStr">
+        <is>
+          <t>MESSAGE_MARKETPLACE_LISTING_RECOVERY_MESSAGE</t>
+        </is>
+      </c>
+      <c r="B39" s="1" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C39" s="1" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D39" s="1" t="inlineStr">
+        <is>
+          <t>거래소 등록이 실패했습니다. 아이템이 통합보관함으로 반환되었습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="inlineStr">
+        <is>
+          <t>MESSAGE_MARKETPLACE_PURCHASE_RECOVERY_TITLE</t>
+        </is>
+      </c>
+      <c r="B40" s="1" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C40" s="1" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D40" s="1" t="inlineStr">
+        <is>
+          <t>거래소 구매 복구</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="inlineStr">
+        <is>
+          <t>MESSAGE_MARKETPLACE_PURCHASE_RECOVERY_MESSAGE</t>
+        </is>
+      </c>
+      <c r="B41" s="1" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C41" s="1" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D41" s="1" t="inlineStr">
+        <is>
+          <t>거래소 구매가 실패했습니다. 돈이 통합보관함으로 반환되었습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="inlineStr">
+        <is>
+          <t>MESSAGE_MARKETPLACE_LISTING_CANCELLED_TITLE</t>
+        </is>
+      </c>
+      <c r="B42" s="1" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C42" s="1" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D42" s="1" t="inlineStr">
+        <is>
+          <t>거래소 등록 취소</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="inlineStr">
+        <is>
+          <t>MESSAGE_MARKETPLACE_LISTING_CANCELLED_MESSAGE</t>
+        </is>
+      </c>
+      <c r="B43" s="1" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C43" s="1" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D43" s="1" t="inlineStr">
+        <is>
+          <t>거래소 등록이 취소되었습니다. 아이템이 통합보관함으로 반환되었습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="inlineStr">
+        <is>
+          <t>MESSAGE_MARKETPLACE_SALE_TITLE</t>
+        </is>
+      </c>
+      <c r="B44" s="1" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C44" s="1" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D44" s="1" t="inlineStr">
+        <is>
+          <t>거래소 판매</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="inlineStr">
+        <is>
+          <t>MESSAGE_MARKETPLACE_SALE_MESSAGE</t>
+        </is>
+      </c>
+      <c r="B45" s="1" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C45" s="1" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D45" s="1" t="inlineStr">
+        <is>
+          <t>아이템이 {}전에 판매되었습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="1" t="inlineStr">
+        <is>
+          <t>MESSAGE_MARKETPLACE_PURCHASE_TITLE</t>
+        </is>
+      </c>
+      <c r="B46" s="1" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C46" s="1" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D46" s="1" t="inlineStr">
+        <is>
+          <t>거래소 구매</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="inlineStr">
+        <is>
+          <t>MESSAGE_MARKETPLACE_PURCHASE_MESSAGE</t>
+        </is>
+      </c>
+      <c r="B47" s="1" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C47" s="1" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D47" s="1" t="inlineStr">
+        <is>
+          <t>거래소에서 아이템을 구매하셨습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="1" t="inlineStr">
+        <is>
+          <t>MESSAGE_NOT_ANY_REPAIRABLE</t>
+        </is>
+      </c>
+      <c r="B48" s="1" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C48" s="1" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D48" s="1" t="inlineStr">
+        <is>
+          <t>고칠 물건이 없습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="1" t="inlineStr">
+        <is>
+          <t>MESSAGE_CANNOT_DEPOSITE_MORE</t>
+        </is>
+      </c>
+      <c r="B49" s="1" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C49" s="1" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D49" s="1" t="inlineStr">
+        <is>
+          <t>더 이상 맡길 수 없습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="1" t="inlineStr">
+        <is>
+          <t>MESSAGE_NOT_DEPOSITED_MONEY</t>
+        </is>
+      </c>
+      <c r="B50" s="1" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C50" s="1" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D50" s="1" t="inlineStr">
+        <is>
+          <t>맡아둔 돈이 없습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="1" t="inlineStr">
+        <is>
+          <t>MESSAGE_NOT_DEPOSITED_ENOUGH</t>
+        </is>
+      </c>
+      <c r="B51" s="1" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C51" s="1" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D51" s="1" t="inlineStr">
+        <is>
+          <t>그만큼 맡기지 않았습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="1" t="inlineStr">
+        <is>
+          <t>MESSAGE_HAVE_MUCH_MONEY</t>
+        </is>
+      </c>
+      <c r="B52" s="1" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C52" s="1" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D52" s="1" t="inlineStr">
+        <is>
+          <t>소지금이 너무 많습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="1" t="inlineStr">
+        <is>
+          <t>MESSAGE_NOT_DEPOSITED_THIS_ITEM</t>
+        </is>
+      </c>
+      <c r="B53" s="1" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C53" s="1" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D53" s="1" t="inlineStr">
+        <is>
+          <t>그런 물품은 맡아두고 있지 않습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="1" t="inlineStr">
+        <is>
+          <t>MESSAGE_UNKNOWN_ERROR</t>
+        </is>
+      </c>
+      <c r="B54" s="1" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C54" s="1" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D54" s="1" t="inlineStr">
+        <is>
+          <t>알 수 없는 에러</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="1" t="inlineStr">
+        <is>
+          <t>MESSAGE_INVALID_ITEM_NAME</t>
+        </is>
+      </c>
+      <c r="B55" s="1" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C55" s="1" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D55" s="1" t="inlineStr">
+        <is>
+          <t>그게 뭐야?</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="1" t="inlineStr">
+        <is>
+          <t>MESSAGE_WEAWPON_NAME_TOO_SHORT</t>
+        </is>
+      </c>
+      <c r="B56" s="1" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C56" s="1" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D56" s="1" t="inlineStr">
+        <is>
+          <t>이름이 너무 짧습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="1" t="inlineStr">
+        <is>
+          <t>MESSAGE_WEAPON_NAME_TOO_LONG</t>
+        </is>
+      </c>
+      <c r="B57" s="1" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C57" s="1" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D57" s="1" t="inlineStr">
+        <is>
+          <t>이름이 너무 깁니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="1" t="inlineStr">
+        <is>
+          <t>MESSAGE_INVALID_WEAPON_NAME</t>
+        </is>
+      </c>
+      <c r="B58" s="1" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C58" s="1" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D58" s="1" t="inlineStr">
+        <is>
+          <t>그렇게 바꿀 수 없습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="1" t="inlineStr">
+        <is>
+          <t>MESSAGE_NO_ANY_DEPOSITED</t>
+        </is>
+      </c>
+      <c r="B59" s="1" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C59" s="1" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D59" s="1" t="inlineStr">
+        <is>
+          <t>맡긴 물건이 없습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="1" t="inlineStr">
+        <is>
+          <t>MESSAGE_NO_ITEM_DEPOSITED</t>
+        </is>
+      </c>
+      <c r="B60" s="1" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C60" s="1" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D60" s="1" t="inlineStr">
+        <is>
+          <t>그런 물건은 맡고 있지 않습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="1" t="inlineStr">
+        <is>
           <t>MESSAGE_NO_RECIPE</t>
         </is>
       </c>
-      <c r="B36" s="1" t="inlineStr">
-        <is>
-          <t>server</t>
-        </is>
-      </c>
-      <c r="C36" s="1" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="D36" s="1" t="inlineStr">
+      <c r="B61" s="1" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C61" s="1" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D61" s="1" t="inlineStr">
         <is>
           <t>조합할 수 없습니다.</t>
         </is>

</xml_diff>

<commit_message>
feat: implement marketplace partial purchase and improve JSON serialization
- Add marketplace_purchase table for partial purchase support
- Replace Json::FastWriter with StreamWriterBuilder for UTF-8 output without escape sequences
- Remove transaction_fee, keep only listing_fee (5%)
- Add purchase_id generation in game server
- Update recovery logic for partial purchases
- Add pre-purchase item condition warnings in Lua
- Add listing fee confirmation dialog
- Set unlimited expiry for marketplace storage_box deliveries
</commit_message>
<xml_diff>
--- a/resources/table/const.string.xlsx
+++ b/resources/table/const.string.xlsx
@@ -4865,7 +4865,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D61"/>
+  <dimension ref="A1:D63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -5779,7 +5779,7 @@
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_MARKETPLACE_LISTING_CANCELLED_TITLE</t>
+          <t>MESSAGE_MARKETPLACE_PURCHASE_REFUND_TITLE</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -5794,14 +5794,14 @@
       </c>
       <c r="D42" s="1" t="inlineStr">
         <is>
-          <t>거래소 등록 취소</t>
+          <t>거래소 구매</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_MARKETPLACE_LISTING_CANCELLED_MESSAGE</t>
+          <t>MESSAGE_MARKETPLACE_PURCHASE_REFUND_MESSAGE</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
@@ -5816,14 +5816,14 @@
       </c>
       <c r="D43" s="1" t="inlineStr">
         <is>
-          <t>거래소 등록이 취소되었습니다. 아이템이 통합보관함으로 반환되었습니다.</t>
+          <t>{} {}개를 {}전에 구매하셨습니다. 요청한 수량보다 적게 구매되어 {}전이 환불되었습니다.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_MARKETPLACE_SALE_TITLE</t>
+          <t>MESSAGE_MARKETPLACE_LISTING_CANCELLED_TITLE</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
@@ -5838,14 +5838,14 @@
       </c>
       <c r="D44" s="1" t="inlineStr">
         <is>
-          <t>거래소 판매</t>
+          <t>거래소 등록 취소</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_MARKETPLACE_SALE_MESSAGE</t>
+          <t>MESSAGE_MARKETPLACE_LISTING_CANCELLED_MESSAGE</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
@@ -5860,14 +5860,14 @@
       </c>
       <c r="D45" s="1" t="inlineStr">
         <is>
-          <t>아이템이 {}전에 판매되었습니다.</t>
+          <t>거래소 등록이 취소되었습니다. 아이템이 통합보관함으로 반환되었습니다.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_MARKETPLACE_PURCHASE_TITLE</t>
+          <t>MESSAGE_MARKETPLACE_SALE_TITLE</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -5882,14 +5882,14 @@
       </c>
       <c r="D46" s="1" t="inlineStr">
         <is>
-          <t>거래소 구매</t>
+          <t>거래소 판매</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_MARKETPLACE_PURCHASE_MESSAGE</t>
+          <t>MESSAGE_MARKETPLACE_SALE_MESSAGE</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -5904,14 +5904,14 @@
       </c>
       <c r="D47" s="1" t="inlineStr">
         <is>
-          <t>거래소에서 아이템을 구매하셨습니다.</t>
+          <t>{} {}개가 {}전에 판매되었습니다.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_NOT_ANY_REPAIRABLE</t>
+          <t>MESSAGE_MARKETPLACE_PURCHASE_TITLE</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -5926,14 +5926,14 @@
       </c>
       <c r="D48" s="1" t="inlineStr">
         <is>
-          <t>고칠 물건이 없습니다.</t>
+          <t>거래소 구매</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_CANNOT_DEPOSITE_MORE</t>
+          <t>MESSAGE_MARKETPLACE_PURCHASE_MESSAGE</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -5948,14 +5948,14 @@
       </c>
       <c r="D49" s="1" t="inlineStr">
         <is>
-          <t>더 이상 맡길 수 없습니다.</t>
+          <t>{} {}개를 {}전에 구매하셨습니다.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_NOT_DEPOSITED_MONEY</t>
+          <t>MESSAGE_NOT_ANY_REPAIRABLE</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -5970,14 +5970,14 @@
       </c>
       <c r="D50" s="1" t="inlineStr">
         <is>
-          <t>맡아둔 돈이 없습니다.</t>
+          <t>고칠 물건이 없습니다.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_NOT_DEPOSITED_ENOUGH</t>
+          <t>MESSAGE_CANNOT_DEPOSITE_MORE</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -5992,14 +5992,14 @@
       </c>
       <c r="D51" s="1" t="inlineStr">
         <is>
-          <t>그만큼 맡기지 않았습니다.</t>
+          <t>더 이상 맡길 수 없습니다.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_HAVE_MUCH_MONEY</t>
+          <t>MESSAGE_NOT_DEPOSITED_MONEY</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -6014,14 +6014,14 @@
       </c>
       <c r="D52" s="1" t="inlineStr">
         <is>
-          <t>소지금이 너무 많습니다.</t>
+          <t>맡아둔 돈이 없습니다.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_NOT_DEPOSITED_THIS_ITEM</t>
+          <t>MESSAGE_NOT_DEPOSITED_ENOUGH</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -6036,14 +6036,14 @@
       </c>
       <c r="D53" s="1" t="inlineStr">
         <is>
-          <t>그런 물품은 맡아두고 있지 않습니다.</t>
+          <t>그만큼 맡기지 않았습니다.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_UNKNOWN_ERROR</t>
+          <t>MESSAGE_HAVE_MUCH_MONEY</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -6058,14 +6058,14 @@
       </c>
       <c r="D54" s="1" t="inlineStr">
         <is>
-          <t>알 수 없는 에러</t>
+          <t>소지금이 너무 많습니다.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_INVALID_ITEM_NAME</t>
+          <t>MESSAGE_NOT_DEPOSITED_THIS_ITEM</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -6080,14 +6080,14 @@
       </c>
       <c r="D55" s="1" t="inlineStr">
         <is>
-          <t>그게 뭐야?</t>
+          <t>그런 물품은 맡아두고 있지 않습니다.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_WEAWPON_NAME_TOO_SHORT</t>
+          <t>MESSAGE_UNKNOWN_ERROR</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -6102,14 +6102,14 @@
       </c>
       <c r="D56" s="1" t="inlineStr">
         <is>
-          <t>이름이 너무 짧습니다.</t>
+          <t>알 수 없는 에러</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_WEAPON_NAME_TOO_LONG</t>
+          <t>MESSAGE_INVALID_ITEM_NAME</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -6124,14 +6124,14 @@
       </c>
       <c r="D57" s="1" t="inlineStr">
         <is>
-          <t>이름이 너무 깁니다.</t>
+          <t>그게 뭐야?</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_INVALID_WEAPON_NAME</t>
+          <t>MESSAGE_WEAWPON_NAME_TOO_SHORT</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -6146,14 +6146,14 @@
       </c>
       <c r="D58" s="1" t="inlineStr">
         <is>
-          <t>그렇게 바꿀 수 없습니다.</t>
+          <t>이름이 너무 짧습니다.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_NO_ANY_DEPOSITED</t>
+          <t>MESSAGE_WEAPON_NAME_TOO_LONG</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -6168,14 +6168,14 @@
       </c>
       <c r="D59" s="1" t="inlineStr">
         <is>
-          <t>맡긴 물건이 없습니다.</t>
+          <t>이름이 너무 깁니다.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_NO_ITEM_DEPOSITED</t>
+          <t>MESSAGE_INVALID_WEAPON_NAME</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
@@ -6190,27 +6190,71 @@
       </c>
       <c r="D60" s="1" t="inlineStr">
         <is>
-          <t>그런 물건은 맡고 있지 않습니다.</t>
+          <t>그렇게 바꿀 수 없습니다.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
+          <t>MESSAGE_NO_ANY_DEPOSITED</t>
+        </is>
+      </c>
+      <c r="B61" s="1" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C61" s="1" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D61" s="1" t="inlineStr">
+        <is>
+          <t>맡긴 물건이 없습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="1" t="inlineStr">
+        <is>
+          <t>MESSAGE_NO_ITEM_DEPOSITED</t>
+        </is>
+      </c>
+      <c r="B62" s="1" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C62" s="1" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D62" s="1" t="inlineStr">
+        <is>
+          <t>그런 물건은 맡고 있지 않습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="1" t="inlineStr">
+        <is>
           <t>MESSAGE_NO_RECIPE</t>
         </is>
       </c>
-      <c r="B61" s="1" t="inlineStr">
-        <is>
-          <t>server</t>
-        </is>
-      </c>
-      <c r="C61" s="1" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="D61" s="1" t="inlineStr">
+      <c r="B63" s="1" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C63" s="1" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D63" s="1" t="inlineStr">
         <is>
           <t>조합할 수 없습니다.</t>
         </is>

</xml_diff>

<commit_message>
feat: add marketplace listing archive system
- Add marketplace_listing_archive table for archiving expired/sold/cancelled listings
- Implement MarketplaceArchiveService for archiving operations
- Add MarketplaceArchiveBackgroundService for periodic archiving
- Add archive-related message constants for expired listings
- Refactor repository structure using DbContext pattern
- Move MarketplaceRepository and MarketplacePurchaseRepository to Marketplace.Reepository namespace
- Update MarketplaceService to use DbContext instead of direct repository injection
- Add code formatting improvements
</commit_message>
<xml_diff>
--- a/resources/table/const.string.xlsx
+++ b/resources/table/const.string.xlsx
@@ -4865,7 +4865,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D63"/>
+  <dimension ref="A1:D66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -5867,7 +5867,7 @@
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_MARKETPLACE_SALE_TITLE</t>
+          <t>MESSAGE_MARKETPLACE_LISTING_EXPIRED_TITLE</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -5882,14 +5882,14 @@
       </c>
       <c r="D46" s="1" t="inlineStr">
         <is>
-          <t>거래소 판매</t>
+          <t>거래소 등록 만료</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_MARKETPLACE_SALE_MESSAGE</t>
+          <t>MESSAGE_MARKETPLACE_LISTING_EXPIRED_MESSAGE</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -5904,14 +5904,14 @@
       </c>
       <c r="D47" s="1" t="inlineStr">
         <is>
-          <t>{} {}개가 {}전에 판매되었습니다.</t>
+          <t>{} {}개가 만료되어 반환되었습니다.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_MARKETPLACE_PURCHASE_TITLE</t>
+          <t>MESSAGE_MARKETPLACE_LISTING_EXPIRED_MESSAGE_WITH_FEE</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -5926,14 +5926,14 @@
       </c>
       <c r="D48" s="1" t="inlineStr">
         <is>
-          <t>거래소 구매</t>
+          <t>{} {}개가 만료되어 반환되었습니다. 등록 수수료 {}전이 함께 반환되었습니다.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_MARKETPLACE_PURCHASE_MESSAGE</t>
+          <t>MESSAGE_MARKETPLACE_SALE_TITLE</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -5948,14 +5948,14 @@
       </c>
       <c r="D49" s="1" t="inlineStr">
         <is>
-          <t>{} {}개를 {}전에 구매하셨습니다.</t>
+          <t>거래소 판매</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_NOT_ANY_REPAIRABLE</t>
+          <t>MESSAGE_MARKETPLACE_SALE_MESSAGE</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -5970,14 +5970,14 @@
       </c>
       <c r="D50" s="1" t="inlineStr">
         <is>
-          <t>고칠 물건이 없습니다.</t>
+          <t>{} {}개가 {}전에 판매되었습니다.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_CANNOT_DEPOSITE_MORE</t>
+          <t>MESSAGE_MARKETPLACE_PURCHASE_TITLE</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -5992,14 +5992,14 @@
       </c>
       <c r="D51" s="1" t="inlineStr">
         <is>
-          <t>더 이상 맡길 수 없습니다.</t>
+          <t>거래소 구매</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_NOT_DEPOSITED_MONEY</t>
+          <t>MESSAGE_MARKETPLACE_PURCHASE_MESSAGE</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -6014,14 +6014,14 @@
       </c>
       <c r="D52" s="1" t="inlineStr">
         <is>
-          <t>맡아둔 돈이 없습니다.</t>
+          <t>{} {}개를 {}전에 구매하셨습니다.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_NOT_DEPOSITED_ENOUGH</t>
+          <t>MESSAGE_NOT_ANY_REPAIRABLE</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -6036,14 +6036,14 @@
       </c>
       <c r="D53" s="1" t="inlineStr">
         <is>
-          <t>그만큼 맡기지 않았습니다.</t>
+          <t>고칠 물건이 없습니다.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_HAVE_MUCH_MONEY</t>
+          <t>MESSAGE_CANNOT_DEPOSITE_MORE</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -6058,14 +6058,14 @@
       </c>
       <c r="D54" s="1" t="inlineStr">
         <is>
-          <t>소지금이 너무 많습니다.</t>
+          <t>더 이상 맡길 수 없습니다.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_NOT_DEPOSITED_THIS_ITEM</t>
+          <t>MESSAGE_NOT_DEPOSITED_MONEY</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -6080,14 +6080,14 @@
       </c>
       <c r="D55" s="1" t="inlineStr">
         <is>
-          <t>그런 물품은 맡아두고 있지 않습니다.</t>
+          <t>맡아둔 돈이 없습니다.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_UNKNOWN_ERROR</t>
+          <t>MESSAGE_NOT_DEPOSITED_ENOUGH</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -6102,14 +6102,14 @@
       </c>
       <c r="D56" s="1" t="inlineStr">
         <is>
-          <t>알 수 없는 에러</t>
+          <t>그만큼 맡기지 않았습니다.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_INVALID_ITEM_NAME</t>
+          <t>MESSAGE_HAVE_MUCH_MONEY</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -6124,14 +6124,14 @@
       </c>
       <c r="D57" s="1" t="inlineStr">
         <is>
-          <t>그게 뭐야?</t>
+          <t>소지금이 너무 많습니다.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_WEAWPON_NAME_TOO_SHORT</t>
+          <t>MESSAGE_NOT_DEPOSITED_THIS_ITEM</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -6146,14 +6146,14 @@
       </c>
       <c r="D58" s="1" t="inlineStr">
         <is>
-          <t>이름이 너무 짧습니다.</t>
+          <t>그런 물품은 맡아두고 있지 않습니다.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_WEAPON_NAME_TOO_LONG</t>
+          <t>MESSAGE_UNKNOWN_ERROR</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -6168,14 +6168,14 @@
       </c>
       <c r="D59" s="1" t="inlineStr">
         <is>
-          <t>이름이 너무 깁니다.</t>
+          <t>알 수 없는 에러</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_INVALID_WEAPON_NAME</t>
+          <t>MESSAGE_INVALID_ITEM_NAME</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
@@ -6190,14 +6190,14 @@
       </c>
       <c r="D60" s="1" t="inlineStr">
         <is>
-          <t>그렇게 바꿀 수 없습니다.</t>
+          <t>그게 뭐야?</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_NO_ANY_DEPOSITED</t>
+          <t>MESSAGE_WEAWPON_NAME_TOO_SHORT</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
@@ -6212,14 +6212,14 @@
       </c>
       <c r="D61" s="1" t="inlineStr">
         <is>
-          <t>맡긴 물건이 없습니다.</t>
+          <t>이름이 너무 짧습니다.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>MESSAGE_NO_ITEM_DEPOSITED</t>
+          <t>MESSAGE_WEAPON_NAME_TOO_LONG</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
@@ -6234,27 +6234,93 @@
       </c>
       <c r="D62" s="1" t="inlineStr">
         <is>
-          <t>그런 물건은 맡고 있지 않습니다.</t>
+          <t>이름이 너무 깁니다.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
+          <t>MESSAGE_INVALID_WEAPON_NAME</t>
+        </is>
+      </c>
+      <c r="B63" s="1" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C63" s="1" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D63" s="1" t="inlineStr">
+        <is>
+          <t>그렇게 바꿀 수 없습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="1" t="inlineStr">
+        <is>
+          <t>MESSAGE_NO_ANY_DEPOSITED</t>
+        </is>
+      </c>
+      <c r="B64" s="1" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C64" s="1" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D64" s="1" t="inlineStr">
+        <is>
+          <t>맡긴 물건이 없습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="1" t="inlineStr">
+        <is>
+          <t>MESSAGE_NO_ITEM_DEPOSITED</t>
+        </is>
+      </c>
+      <c r="B65" s="1" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C65" s="1" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D65" s="1" t="inlineStr">
+        <is>
+          <t>그런 물건은 맡고 있지 않습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="1" t="inlineStr">
+        <is>
           <t>MESSAGE_NO_RECIPE</t>
         </is>
       </c>
-      <c r="B63" s="1" t="inlineStr">
-        <is>
-          <t>server</t>
-        </is>
-      </c>
-      <c r="C63" s="1" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="D63" s="1" t="inlineStr">
+      <c r="B66" s="1" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C66" s="1" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D66" s="1" t="inlineStr">
         <is>
           <t>조합할 수 없습니다.</t>
         </is>

</xml_diff>

<commit_message>
feat: add not repairable message and bot skip redundant updates
- Add MESSAGE_ITEM_NOT_REPAIRABLE to model and const.string table
- Bot: skip change_level/change_stats/change_str/change_dex/change_int when value unchanged
- Update Pulumi config (admin-tool, internal, marketplace, mysql, rabbitmq, redis, write-back)
- Update HTTP services (Bulletin, Session, Cache, DbContext, Log, ServerState, Storage, WriteBack, ShutdownListener)
- Update BulletinController, GroupService, gateway server, admin-tool Auth/User services
- Update game character, server.bulletin, interaction.lua, npc.lua
- Update Model.cs, Repository.Achievement, marketplace DbContext

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/resources/table/const.string.xlsx
+++ b/resources/table/const.string.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\fb\resources\table\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CAE72A0-E733-42A3-9BCA-32683B7E96AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6E1C3EF-F81C-4504-81AA-556EE42EC811}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="5" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="string.game.asset" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1044" uniqueCount="520">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1048" uniqueCount="522">
   <si>
     <t>MESSAGE_ASSET_MAP_LOADED</t>
   </si>
@@ -1604,6 +1604,14 @@
   </si>
   <si>
     <t>예상 종료 시간: {}</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>MESSAGE_ITEM_NOT_REPAIRABLE</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>고칠 물건이 없습니다.</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -1667,7 +1675,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -2912,7 +2920,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -3035,7 +3043,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>405</v>
+        <v>520</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>1</v>
@@ -3044,12 +3052,12 @@
         <v>2</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>406</v>
+        <v>521</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>1</v>
@@ -3058,20 +3066,34 @@
         <v>2</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
+        <v>407</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
         <v>409</v>
       </c>
-      <c r="B11" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D11" s="1" t="s">
+      <c r="B12" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D12" s="1" t="s">
         <v>410</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: migrate game scripts to numeric IDs and harden Lua loading
- Rename spell, item, npc, and mob scripts to model ID paths
- Add Lua context guard and safer load or execute return values
- Initialize map scripts on server startup and update script loader
- Update game data tables, model bindings, and C++ script hooks
- Validate nation, gender, and creature on character creation
- Fix quest map IDs and mountain treasure handler order
- Update bot integration tests for script path changes
</commit_message>
<xml_diff>
--- a/resources/table/const.string.xlsx
+++ b/resources/table/const.string.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6E1C3EF-F81C-4504-81AA-556EE42EC811}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39B12B90-42A4-4353-A89D-DED23440F62F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="5" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="14" activeTab="19" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="string.game.asset" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1048" uniqueCount="522">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1056" uniqueCount="526">
   <si>
     <t>MESSAGE_ASSET_MAP_LOADED</t>
   </si>
@@ -1613,6 +1613,18 @@
   <si>
     <t>고칠 물건이 없습니다.</t>
     <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>MESSAGE_CLIENT_GENDER_INVALID</t>
+  </si>
+  <si>
+    <t>MESSAGE_CLIENT_CREATURE_INVALID</t>
+  </si>
+  <si>
+    <t>성별이 올바르지 않습니다.</t>
+  </si>
+  <si>
+    <t>수호신이 올바르지 않습니다.</t>
   </si>
 </sst>
 </file>
@@ -3888,16 +3900,17 @@
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1300-000000000000}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="40" customWidth="1"/>
-    <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="10" customWidth="1"/>
-    <col min="4" max="4" width="60" customWidth="1"/>
+    <col min="1" max="1" width="40" style="2" customWidth="1"/>
+    <col min="2" max="2" width="12" style="2" customWidth="1"/>
+    <col min="3" max="3" width="10" style="2" customWidth="1"/>
+    <col min="4" max="4" width="60" style="2" customWidth="1"/>
+    <col min="5" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>480</v>
       </c>
@@ -3911,7 +3924,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>482</v>
       </c>
@@ -3923,6 +3936,34 @@
       </c>
       <c r="D2" s="1" t="s">
         <v>483</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>522</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>523</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>525</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: block non-tradeable items from marketplace listing
- Add MARKETPLACE_ITEM_NOT_TRADEABLE error code and register-item message
- Validate item trade flag in game server, Lua UI, and marketplace service
- Expose model:trade() Lua binding for item models
</commit_message>
<xml_diff>
--- a/resources/table/const.string.xlsx
+++ b/resources/table/const.string.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39B12B90-42A4-4353-A89D-DED23440F62F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{321FEAFA-97BC-431A-98C7-E5E6E0B140C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="14" activeTab="19" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="8" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="string.game.asset" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1056" uniqueCount="526">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1060" uniqueCount="528">
   <si>
     <t>MESSAGE_ASSET_MAP_LOADED</t>
   </si>
@@ -1625,6 +1625,14 @@
   </si>
   <si>
     <t>수호신이 올바르지 않습니다.</t>
+  </si>
+  <si>
+    <t>MESSAGE_EXCEPTION_CANNOT_REGISTER_ITEM</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>등록할 수 없는 물건입니다.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -5899,16 +5907,17 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:D9"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:D10"/>
+  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="40" customWidth="1"/>
-    <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="10" customWidth="1"/>
-    <col min="4" max="4" width="60" customWidth="1"/>
+    <col min="1" max="1" width="40" style="2" customWidth="1"/>
+    <col min="2" max="2" width="12" style="2" customWidth="1"/>
+    <col min="3" max="3" width="10" style="2" customWidth="1"/>
+    <col min="4" max="4" width="60" style="2" customWidth="1"/>
+    <col min="5" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>340</v>
       </c>
@@ -5922,7 +5931,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>342</v>
       </c>
@@ -5936,7 +5945,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>344</v>
       </c>
@@ -5950,7 +5959,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>346</v>
       </c>
@@ -5964,7 +5973,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>348</v>
       </c>
@@ -5978,7 +5987,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>350</v>
       </c>
@@ -5992,7 +6001,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>352</v>
       </c>
@@ -6006,7 +6015,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>354</v>
       </c>
@@ -6020,7 +6029,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>356</v>
       </c>
@@ -6032,6 +6041,20 @@
       </c>
       <c r="D9" s="1" t="s">
         <v>357</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>526</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>515</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>516</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>527</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: implement friend system with mutual sync
- Add friend table, repository, and FriendService with distributed locks
- Mirror client friend list via Init/UpdateFriends and AMQP peer updates
- Support mutual-only !!! chat and login notifications
- Add friend-related protocol messages and string resources
</commit_message>
<xml_diff>
--- a/resources/table/const.string.xlsx
+++ b/resources/table/const.string.xlsx
@@ -4013,7 +4013,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -4547,6 +4547,28 @@
       <c r="D24" t="inlineStr">
         <is>
           <t>대상 문파를 찾을 수 없습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>MESSAGE_CLAN_NOT_JOINED</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>문파에 가입하지 않았습니다.</t>
         </is>
       </c>
     </row>
@@ -4561,7 +4583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -4633,6 +4655,50 @@
       <c r="D3" s="1" t="inlineStr">
         <is>
           <t>귓속말을 할 수 없는 지역입니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>MESSAGE_FRIEND_CHAT_NO_MUTUAL</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>상호 친구가 없습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>MESSAGE_FRIEND_LOGIN</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>[친구] {}님이 접속하셨습니다.</t>
         </is>
       </c>
     </row>

</xml_diff>